<commit_message>
Corrected refresh: 2 verified new listings (Hightouch, Typeform) after manual board verification
</commit_message>
<xml_diff>
--- a/Remote_Job_Search_Tracker.xlsx
+++ b/Remote_Job_Search_Tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3106,6 +3106,146 @@
       <c r="P34" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">10+ Years of relevant experience </t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Customer Success Engineer</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Hightouch</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Customer Success</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Anywhere in the World (platform tag)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>$85,000-$110,000 (well above target)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Salary far above target - listing includes an E-Verify statement, which usually signals US work-authorization requirement despite the 'Anywhere in the World' tag. Verify on application before investing time.</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>We Work Remotely</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/hightouch-customer-success-engineer</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Apply via WWR listing</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>To Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Customer Success Manager</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Typeform</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Customer Success</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Anywhere in the World (platform tag)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>$65,000-$95,000 (above target)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Listing says they're 'especially excited to hire someone based in the ET Timezone' - real-time overlap with US Eastern would be tough from Riyadh; worth a shot but deprioritize timezone-heavy expectations.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>We Work Remotely</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/typeform-customer-success-manager</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Apply via WWR listing</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>To Review</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3325,7 @@
         </is>
       </c>
       <c r="B3" s="10">
-        <f>COUNTA('Job Tracker'!B2:B34)</f>
+        <f>COUNTA('Job Tracker'!B2:B36)</f>
         <v/>
       </c>
     </row>
@@ -3196,7 +3336,7 @@
         </is>
       </c>
       <c r="B4" s="10">
-        <f>COUNTIF('Job Tracker'!G2:G34,"High")</f>
+        <f>COUNTIF('Job Tracker'!G2:G36,"High")</f>
         <v/>
       </c>
     </row>
@@ -3207,7 +3347,7 @@
         </is>
       </c>
       <c r="B5" s="10">
-        <f>COUNTIF('Job Tracker'!G2:G34,"Medium")</f>
+        <f>COUNTIF('Job Tracker'!G2:G36,"Medium")</f>
         <v/>
       </c>
     </row>
@@ -3218,7 +3358,7 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>COUNTIF('Job Tracker'!G2:G34,"Low")</f>
+        <f>COUNTIF('Job Tracker'!G2:G36,"Low")</f>
         <v/>
       </c>
     </row>
@@ -3229,7 +3369,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>COUNTIF('Job Tracker'!N2:N34,"Applied")</f>
+        <f>COUNTIF('Job Tracker'!N2:N36,"Applied")</f>
         <v/>
       </c>
     </row>
@@ -3240,7 +3380,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>COUNTIF('Job Tracker'!N2:N34,"Interview")</f>
+        <f>COUNTIF('Job Tracker'!N2:N36,"Interview")</f>
         <v/>
       </c>
     </row>
@@ -3251,7 +3391,7 @@
         </is>
       </c>
       <c r="B9" s="10">
-        <f>COUNTIF('Job Tracker'!N2:N34,"Offer")</f>
+        <f>COUNTIF('Job Tracker'!N2:N36,"Offer")</f>
         <v/>
       </c>
     </row>
@@ -3262,7 +3402,7 @@
         </is>
       </c>
       <c r="B10" s="10">
-        <f>COUNTIF('Job Tracker'!N2:N34,"To Review")</f>
+        <f>COUNTIF('Job Tracker'!N2:N36,"To Review")</f>
         <v/>
       </c>
     </row>
@@ -3280,7 +3420,7 @@
         </is>
       </c>
       <c r="B14" s="10">
-        <f>COUNTIF('Job Tracker'!D2:D34,"TAM")</f>
+        <f>COUNTIF('Job Tracker'!D2:D36,"TAM")</f>
         <v/>
       </c>
     </row>
@@ -3291,7 +3431,7 @@
         </is>
       </c>
       <c r="B15" s="10">
-        <f>COUNTIF('Job Tracker'!D2:D34,"Customer Success")</f>
+        <f>COUNTIF('Job Tracker'!D2:D36,"Customer Success")</f>
         <v/>
       </c>
     </row>
@@ -3302,7 +3442,7 @@
         </is>
       </c>
       <c r="B16" s="10">
-        <f>COUNTIF('Job Tracker'!D2:D34,"Solution Consultant")</f>
+        <f>COUNTIF('Job Tracker'!D2:D36,"Solution Consultant")</f>
         <v/>
       </c>
     </row>
@@ -3313,7 +3453,7 @@
         </is>
       </c>
       <c r="B17" s="10">
-        <f>COUNTIF('Job Tracker'!D2:D34,"Application Support")</f>
+        <f>COUNTIF('Job Tracker'!D2:D36,"Application Support")</f>
         <v/>
       </c>
     </row>
@@ -3456,7 +3596,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Refreshed on 2026-08-17. Each run only pulls postings dated within the last 3 days -</t>
+          <t>Refreshed on 2026-08-17 (corrected pass - initial automated refresh under-searched; verified directly against board pages).</t>
         </is>
       </c>
     </row>

</xml_diff>